<commit_message>
Changed board layout and few critical improvements in routing
</commit_message>
<xml_diff>
--- a/BOM_ESP32 SD Interrupter_PCB_PCB_ESP32-sd-int_2026-03-25.xlsx
+++ b/BOM_ESP32 SD Interrupter_PCB_PCB_ESP32-sd-int_2026-03-25.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="229">
   <si>
     <t>No.</t>
   </si>
@@ -292,7 +292,7 @@
     <t>15</t>
   </si>
   <si>
-    <t>FT10MHNR_C17216617</t>
+    <t>HFBR-1521Z</t>
   </si>
   <si>
     <t>OPTO1</t>
@@ -301,13 +301,10 @@
     <t>CONN-TH_HFBR-1521Z</t>
   </si>
   <si>
-    <t>FT10MHNR</t>
-  </si>
-  <si>
-    <t>Firecomms</t>
-  </si>
-  <si>
-    <t>C17216617</t>
+    <t>Broadcom(博通)</t>
+  </si>
+  <si>
+    <t>C188712</t>
   </si>
   <si>
     <t>16</t>
@@ -547,19 +544,25 @@
     <t>TS-1088-AR02016</t>
   </si>
   <si>
-    <t>SW5,SW6</t>
+    <t>SW5</t>
   </si>
   <si>
     <t>SW-SMD_L3.9-W3.0-P4.45</t>
   </si>
   <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>SW6</t>
+  </si>
+  <si>
     <t>XUNPU(讯普)</t>
   </si>
   <si>
     <t>C720477</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>SD</t>
@@ -574,7 +577,7 @@
     <t>C9900023771</t>
   </si>
   <si>
-    <t>31</t>
+    <t>32</t>
   </si>
   <si>
     <t>LESD5D5.0CT1G_C5246195</t>
@@ -595,7 +598,7 @@
     <t>C5246195</t>
   </si>
   <si>
-    <t>32</t>
+    <t>33</t>
   </si>
   <si>
     <t>AMS1117-3.3</t>
@@ -613,7 +616,7 @@
     <t>C6186</t>
   </si>
   <si>
-    <t>33</t>
+    <t>34</t>
   </si>
   <si>
     <t>AMS1117-5.0</t>
@@ -628,7 +631,7 @@
     <t>C6187</t>
   </si>
   <si>
-    <t>34</t>
+    <t>35</t>
   </si>
   <si>
     <t>ESP32-S3-WROOM-1(N8R8)</t>
@@ -649,7 +652,7 @@
     <t>C2913201</t>
   </si>
   <si>
-    <t>35</t>
+    <t>36</t>
   </si>
   <si>
     <t>MIDIJACK</t>
@@ -661,7 +664,7 @@
     <t>CP-2350</t>
   </si>
   <si>
-    <t>36</t>
+    <t>37</t>
   </si>
   <si>
     <t>H11L1</t>
@@ -679,7 +682,7 @@
     <t>C78588</t>
   </si>
   <si>
-    <t>37</t>
+    <t>38</t>
   </si>
   <si>
     <t>MUP-U20409-2</t>
@@ -1071,7 +1074,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="11" width="20" customWidth="1"/>
@@ -1622,13 +1625,13 @@
         <v>15</v>
       </c>
       <c r="G16" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" t="s">
         <v>96</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>97</v>
-      </c>
-      <c r="I16" t="s">
-        <v>98</v>
       </c>
       <c r="J16" t="s">
         <v>19</v>
@@ -1639,776 +1642,811 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
         <v>99</v>
       </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>100</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>101</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" t="s">
+        <v>99</v>
+      </c>
+      <c r="H17" t="s">
         <v>102</v>
       </c>
-      <c r="F17" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" t="s">
-        <v>100</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>103</v>
       </c>
-      <c r="I17" t="s">
-        <v>104</v>
-      </c>
       <c r="J17" t="s">
         <v>19</v>
       </c>
       <c r="K17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" t="s">
         <v>106</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>107</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" t="s">
         <v>108</v>
       </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>109</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>110</v>
       </c>
-      <c r="I18" t="s">
-        <v>111</v>
-      </c>
       <c r="J18" t="s">
         <v>19</v>
       </c>
       <c r="K18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B19">
         <v>2</v>
       </c>
       <c r="C19" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" t="s">
         <v>113</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
+        <v>107</v>
+      </c>
+      <c r="F19" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" t="s">
         <v>114</v>
       </c>
-      <c r="E19" t="s">
-        <v>108</v>
-      </c>
-      <c r="F19" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>115</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>116</v>
       </c>
-      <c r="I19" t="s">
-        <v>117</v>
-      </c>
       <c r="J19" t="s">
         <v>19</v>
       </c>
       <c r="K19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>117</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>118</v>
       </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>119</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
+        <v>107</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" t="s">
         <v>120</v>
       </c>
-      <c r="E20" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>121</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>122</v>
       </c>
-      <c r="I20" t="s">
-        <v>123</v>
-      </c>
       <c r="J20" t="s">
         <v>19</v>
       </c>
       <c r="K20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>124</v>
       </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>125</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
+        <v>107</v>
+      </c>
+      <c r="F21" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" t="s">
         <v>126</v>
       </c>
-      <c r="E21" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>127</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>128</v>
       </c>
-      <c r="I21" t="s">
-        <v>129</v>
-      </c>
       <c r="J21" t="s">
         <v>19</v>
       </c>
       <c r="K21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>130</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>131</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
+        <v>107</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" t="s">
         <v>132</v>
       </c>
-      <c r="E22" t="s">
-        <v>108</v>
-      </c>
-      <c r="F22" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>133</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>134</v>
       </c>
-      <c r="I22" t="s">
-        <v>135</v>
-      </c>
       <c r="J22" t="s">
         <v>19</v>
       </c>
       <c r="K22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>135</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>136</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>137</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>107</v>
+      </c>
+      <c r="F23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" t="s">
         <v>138</v>
       </c>
-      <c r="E23" t="s">
-        <v>108</v>
-      </c>
-      <c r="F23" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>139</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>140</v>
       </c>
-      <c r="I23" t="s">
-        <v>141</v>
-      </c>
       <c r="J23" t="s">
         <v>19</v>
       </c>
       <c r="K23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>142</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>143</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
         <v>144</v>
       </c>
-      <c r="E24" t="s">
-        <v>108</v>
-      </c>
-      <c r="F24" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>145</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>146</v>
       </c>
-      <c r="I24" t="s">
-        <v>147</v>
-      </c>
       <c r="J24" t="s">
         <v>19</v>
       </c>
       <c r="K24" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>148</v>
       </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>149</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" t="s">
         <v>150</v>
       </c>
-      <c r="E25" t="s">
-        <v>108</v>
-      </c>
-      <c r="F25" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
+        <v>145</v>
+      </c>
+      <c r="I25" t="s">
         <v>151</v>
       </c>
-      <c r="H25" t="s">
-        <v>146</v>
-      </c>
-      <c r="I25" t="s">
-        <v>152</v>
-      </c>
       <c r="J25" t="s">
         <v>19</v>
       </c>
       <c r="K25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>152</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>153</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>154</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
+        <v>107</v>
+      </c>
+      <c r="F26" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
         <v>155</v>
       </c>
-      <c r="E26" t="s">
-        <v>108</v>
-      </c>
-      <c r="F26" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
+        <v>145</v>
+      </c>
+      <c r="I26" t="s">
         <v>156</v>
       </c>
-      <c r="H26" t="s">
-        <v>146</v>
-      </c>
-      <c r="I26" t="s">
-        <v>157</v>
-      </c>
       <c r="J26" t="s">
         <v>19</v>
       </c>
       <c r="K26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B27">
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D27" t="s">
+        <v>158</v>
+      </c>
+      <c r="E27" t="s">
         <v>159</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
+        <v>15</v>
+      </c>
+      <c r="G27" t="s">
         <v>160</v>
       </c>
-      <c r="F27" t="s">
-        <v>15</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>161</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>162</v>
       </c>
-      <c r="I27" t="s">
-        <v>163</v>
-      </c>
       <c r="J27" t="s">
         <v>19</v>
       </c>
       <c r="K27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B28">
         <v>3</v>
       </c>
       <c r="C28" t="s">
+        <v>164</v>
+      </c>
+      <c r="D28" t="s">
         <v>165</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>166</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
+        <v>15</v>
+      </c>
+      <c r="G28" t="s">
+        <v>164</v>
+      </c>
+      <c r="H28" t="s">
         <v>167</v>
       </c>
-      <c r="F28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" t="s">
-        <v>165</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>168</v>
       </c>
-      <c r="I28" t="s">
-        <v>169</v>
-      </c>
       <c r="J28" t="s">
         <v>19</v>
       </c>
       <c r="K28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>169</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
         <v>170</v>
       </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>171</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>172</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" t="s">
+        <v>170</v>
+      </c>
+      <c r="H29" t="s">
         <v>173</v>
       </c>
-      <c r="F29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" t="s">
-        <v>171</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>174</v>
       </c>
-      <c r="I29" t="s">
-        <v>175</v>
-      </c>
       <c r="J29" t="s">
         <v>19</v>
       </c>
       <c r="K29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>175</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
         <v>176</v>
       </c>
-      <c r="B30">
-        <v>2</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>177</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>178</v>
       </c>
-      <c r="E30" t="s">
-        <v>179</v>
-      </c>
       <c r="F30" t="s">
         <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>177</v>
+        <v>16</v>
       </c>
       <c r="H30" t="s">
-        <v>180</v>
+        <v>17</v>
       </c>
       <c r="I30" t="s">
-        <v>181</v>
+        <v>18</v>
       </c>
       <c r="J30" t="s">
         <v>19</v>
       </c>
       <c r="K30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>176</v>
+      </c>
+      <c r="D31" t="s">
+        <v>180</v>
+      </c>
+      <c r="E31" t="s">
+        <v>178</v>
+      </c>
+      <c r="F31" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" t="s">
+        <v>176</v>
+      </c>
+      <c r="H31" t="s">
+        <v>181</v>
+      </c>
+      <c r="I31" t="s">
         <v>182</v>
       </c>
-      <c r="B31">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
-        <v>183</v>
-      </c>
-      <c r="D31" t="s">
-        <v>184</v>
-      </c>
-      <c r="E31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" t="s">
-        <v>183</v>
-      </c>
-      <c r="H31" t="s">
-        <v>59</v>
-      </c>
-      <c r="I31" t="s">
-        <v>186</v>
-      </c>
       <c r="J31" t="s">
         <v>19</v>
       </c>
       <c r="K31" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>183</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>184</v>
+      </c>
+      <c r="D32" t="s">
+        <v>185</v>
+      </c>
+      <c r="E32" t="s">
+        <v>186</v>
+      </c>
+      <c r="F32" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" t="s">
+        <v>184</v>
+      </c>
+      <c r="H32" t="s">
+        <v>59</v>
+      </c>
+      <c r="I32" t="s">
         <v>187</v>
       </c>
-      <c r="B32">
-        <v>2</v>
-      </c>
-      <c r="C32" t="s">
-        <v>188</v>
-      </c>
-      <c r="D32" t="s">
-        <v>189</v>
-      </c>
-      <c r="E32" t="s">
-        <v>190</v>
-      </c>
-      <c r="F32" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" t="s">
-        <v>191</v>
-      </c>
-      <c r="H32" t="s">
-        <v>192</v>
-      </c>
-      <c r="I32" t="s">
-        <v>193</v>
-      </c>
       <c r="J32" t="s">
         <v>19</v>
       </c>
       <c r="K32" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>189</v>
+      </c>
+      <c r="D33" t="s">
+        <v>190</v>
+      </c>
+      <c r="E33" t="s">
+        <v>191</v>
+      </c>
+      <c r="F33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G33" t="s">
+        <v>192</v>
+      </c>
+      <c r="H33" t="s">
+        <v>193</v>
+      </c>
+      <c r="I33" t="s">
         <v>194</v>
       </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
-      <c r="C33" t="s">
-        <v>195</v>
-      </c>
-      <c r="D33" t="s">
-        <v>196</v>
-      </c>
-      <c r="E33" t="s">
-        <v>197</v>
-      </c>
-      <c r="F33" t="s">
-        <v>15</v>
-      </c>
-      <c r="G33" t="s">
-        <v>195</v>
-      </c>
-      <c r="H33" t="s">
-        <v>198</v>
-      </c>
-      <c r="I33" t="s">
-        <v>199</v>
-      </c>
       <c r="J33" t="s">
         <v>19</v>
       </c>
       <c r="K33" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>196</v>
+      </c>
+      <c r="D34" t="s">
+        <v>197</v>
+      </c>
+      <c r="E34" t="s">
+        <v>198</v>
+      </c>
+      <c r="F34" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" t="s">
+        <v>196</v>
+      </c>
+      <c r="H34" t="s">
+        <v>199</v>
+      </c>
+      <c r="I34" t="s">
         <v>200</v>
       </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s">
-        <v>201</v>
-      </c>
-      <c r="D34" t="s">
-        <v>202</v>
-      </c>
-      <c r="E34" t="s">
-        <v>203</v>
-      </c>
-      <c r="F34" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" t="s">
-        <v>201</v>
-      </c>
-      <c r="H34" t="s">
-        <v>198</v>
-      </c>
-      <c r="I34" t="s">
-        <v>204</v>
-      </c>
       <c r="J34" t="s">
         <v>19</v>
       </c>
       <c r="K34" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>201</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>202</v>
+      </c>
+      <c r="D35" t="s">
+        <v>203</v>
+      </c>
+      <c r="E35" t="s">
+        <v>204</v>
+      </c>
+      <c r="F35" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" t="s">
+        <v>202</v>
+      </c>
+      <c r="H35" t="s">
+        <v>199</v>
+      </c>
+      <c r="I35" t="s">
         <v>205</v>
       </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>206</v>
-      </c>
-      <c r="D35" t="s">
-        <v>207</v>
-      </c>
-      <c r="E35" t="s">
-        <v>208</v>
-      </c>
-      <c r="F35" t="s">
-        <v>15</v>
-      </c>
-      <c r="G35" t="s">
-        <v>209</v>
-      </c>
-      <c r="H35" t="s">
-        <v>210</v>
-      </c>
-      <c r="I35" t="s">
-        <v>211</v>
-      </c>
       <c r="J35" t="s">
         <v>19</v>
       </c>
       <c r="K35" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>206</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>207</v>
+      </c>
+      <c r="D36" t="s">
+        <v>208</v>
+      </c>
+      <c r="E36" t="s">
+        <v>209</v>
+      </c>
+      <c r="F36" t="s">
+        <v>15</v>
+      </c>
+      <c r="G36" t="s">
+        <v>210</v>
+      </c>
+      <c r="H36" t="s">
+        <v>211</v>
+      </c>
+      <c r="I36" t="s">
         <v>212</v>
       </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>213</v>
-      </c>
-      <c r="D36" t="s">
-        <v>214</v>
-      </c>
-      <c r="E36" t="s">
-        <v>215</v>
-      </c>
-      <c r="F36" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s">
-        <v>15</v>
-      </c>
-      <c r="I36" t="s">
-        <v>15</v>
-      </c>
       <c r="J36" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K36" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>213</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>214</v>
+      </c>
+      <c r="D37" t="s">
+        <v>215</v>
+      </c>
+      <c r="E37" t="s">
         <v>216</v>
       </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-      <c r="C37" t="s">
-        <v>217</v>
-      </c>
-      <c r="D37" t="s">
-        <v>218</v>
-      </c>
-      <c r="E37" t="s">
-        <v>219</v>
-      </c>
       <c r="F37" t="s">
         <v>15</v>
       </c>
       <c r="G37" t="s">
-        <v>217</v>
+        <v>15</v>
       </c>
       <c r="H37" t="s">
-        <v>220</v>
+        <v>15</v>
       </c>
       <c r="I37" t="s">
-        <v>221</v>
+        <v>15</v>
       </c>
       <c r="J37" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="K37" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>217</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>218</v>
+      </c>
+      <c r="D38" t="s">
+        <v>219</v>
+      </c>
+      <c r="E38" t="s">
+        <v>220</v>
+      </c>
+      <c r="F38" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" t="s">
+        <v>218</v>
+      </c>
+      <c r="H38" t="s">
+        <v>221</v>
+      </c>
+      <c r="I38" t="s">
         <v>222</v>
       </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="J38" t="s">
+        <v>19</v>
+      </c>
+      <c r="K38" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>223</v>
       </c>
-      <c r="D38" t="s">
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
         <v>224</v>
       </c>
-      <c r="E38" t="s">
+      <c r="D39" t="s">
         <v>225</v>
       </c>
-      <c r="F38" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" t="s">
-        <v>223</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="E39" t="s">
         <v>226</v>
       </c>
-      <c r="I38" t="s">
+      <c r="F39" t="s">
+        <v>15</v>
+      </c>
+      <c r="G39" t="s">
+        <v>224</v>
+      </c>
+      <c r="H39" t="s">
         <v>227</v>
       </c>
-      <c r="J38" t="s">
-        <v>19</v>
-      </c>
-      <c r="K38" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="I39" t="s">
+        <v>228</v>
+      </c>
+      <c r="J39" t="s">
+        <v>19</v>
+      </c>
+      <c r="K39" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>